<commit_message>
VLOOKUP and INDEX_MATCH functions
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,22 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e56c63efceb36ea0/Desktop/Adv_Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="13_ncr:1_{BF38CFA4-3C87-4133-BF5D-E6AC723716A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDDF1DE4-E87F-4A2C-B006-B6A4DEE6FE0D}"/>
+  <xr:revisionPtr revIDLastSave="699" documentId="13_ncr:1_{BF38CFA4-3C87-4133-BF5D-E6AC723716A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96E7DEAB-E3B4-4567-A635-669B7AFE6B28}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMartDataSet" sheetId="1" r:id="rId1"/>
     <sheet name="FlashFill" sheetId="3" r:id="rId2"/>
     <sheet name="Custom_List" sheetId="4" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="7" r:id="rId5"/>
-    <sheet name="Sheet5" sheetId="5" r:id="rId6"/>
+    <sheet name="Vlookp" sheetId="8" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Custom_List!$B$2:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Sheet2!$D$3:$D$9</definedName>
     <definedName name="Category">DMart_Sales_data[Category]</definedName>
+    <definedName name="Delivery_Date">DMart_Sales_data[delivery_date]</definedName>
     <definedName name="Discount">DMart_Sales_data[discount]</definedName>
+    <definedName name="Order_date">DMart_Sales_data[order_date]</definedName>
     <definedName name="Orders">DMart_Sales_data[OrderID]</definedName>
     <definedName name="Region">DMart_Sales_data[updated_region]</definedName>
     <definedName name="Sales">DMart_Sales_data[sales]</definedName>
@@ -40,14 +44,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -69,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4225" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4271" uniqueCount="717">
   <si>
     <t>Region</t>
   </si>
@@ -2157,6 +2161,69 @@
   </si>
   <si>
     <t>Count of sales for customer type member and payment mode is UPI or Card</t>
+  </si>
+  <si>
+    <t>Total Sales By North</t>
+  </si>
+  <si>
+    <t>Total Sales By South</t>
+  </si>
+  <si>
+    <t>Total Sales By East</t>
+  </si>
+  <si>
+    <t>Total Sales By West</t>
+  </si>
+  <si>
+    <t>Count Sales By North</t>
+  </si>
+  <si>
+    <t>Count Sales By South</t>
+  </si>
+  <si>
+    <t>Count Sales By East</t>
+  </si>
+  <si>
+    <t>Count Sales By West</t>
+  </si>
+  <si>
+    <t>Total sales for 2023</t>
+  </si>
+  <si>
+    <t>Total sales for last 6 months</t>
+  </si>
+  <si>
+    <t>MAX DATE</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Find Duplicates if Employee ID</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Total sales</t>
+  </si>
+  <si>
+    <t>EmplID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Employee ID </t>
+  </si>
+  <si>
+    <t>Match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales </t>
+  </si>
+  <si>
+    <t>Employee Id</t>
+  </si>
+  <si>
+    <t>INDEX-MATCH</t>
   </si>
 </sst>
 </file>
@@ -2168,11 +2235,18 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2293,7 +2367,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2327,6 +2401,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4F4F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2519,61 +2605,61 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
@@ -2582,28 +2668,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="44" fontId="15" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="16" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="60% - Accent4" xfId="2" builtinId="44"/>
@@ -3452,8 +3547,11 @@
     <col min="19" max="19" width="14.44140625" customWidth="1"/>
     <col min="20" max="20" width="8.6640625" customWidth="1"/>
     <col min="21" max="21" width="37.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="26" width="8.6640625" customWidth="1"/>
+    <col min="22" max="22" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.6640625" customWidth="1"/>
+    <col min="24" max="24" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -3577,8 +3675,6 @@
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
-      <c r="X2" s="1"/>
-      <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
       <c r="AB2" s="1"/>
@@ -3714,8 +3810,13 @@
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="1"/>
+      <c r="X4" s="50" t="s">
+        <v>704</v>
+      </c>
+      <c r="Y4" s="57" cm="1">
+        <f t="array" ref="Y4">SUMIF(Order_date,"&lt;2024-01-01",Sales)</f>
+        <v>654586.69000000018</v>
+      </c>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
@@ -3784,8 +3885,13 @@
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="1"/>
+      <c r="X5" s="50" t="s">
+        <v>705</v>
+      </c>
+      <c r="Y5" s="57" cm="1">
+        <f t="array" ref="Y5">SUMIFS(Sales,Order_date,"&lt;=2024-12-31",Order_date,"&gt;2024-06-30")</f>
+        <v>368049.34999999992</v>
+      </c>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
       <c r="AB5" s="1"/>
@@ -3854,8 +3960,13 @@
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
+      <c r="X6" s="56" t="s">
+        <v>705</v>
+      </c>
+      <c r="Y6" s="59" cm="1">
+        <f t="array" ref="Y6">SUMIF(Order_date,"&gt;=2024-07-01",Sales)</f>
+        <v>368049.34999999992</v>
+      </c>
       <c r="Z6" s="1"/>
       <c r="AA6" s="1"/>
       <c r="AB6" s="1"/>
@@ -3982,8 +4093,13 @@
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="1"/>
+      <c r="X8" s="50" t="s">
+        <v>706</v>
+      </c>
+      <c r="Y8" s="62">
+        <f>MAX(Order_date)</f>
+        <v>45657</v>
+      </c>
       <c r="Z8" s="1"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="1"/>
@@ -4124,7 +4240,9 @@
         <v>79466.449999999983</v>
       </c>
       <c r="W10" s="1"/>
-      <c r="X10" s="1"/>
+      <c r="X10" s="56" t="s">
+        <v>710</v>
+      </c>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
       <c r="AA10" s="1"/>
@@ -4991,11 +5109,14 @@
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="1"/>
+      <c r="U22" s="50" t="s">
+        <v>696</v>
+      </c>
+      <c r="V22" s="57" cm="1">
+        <f t="array" ref="V22">SUMIF(Region,"North",Sales)</f>
+        <v>334964.16000000003</v>
+      </c>
       <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
       <c r="AA22" s="1"/>
       <c r="AB22" s="1"/>
@@ -5061,11 +5182,14 @@
         <v>36091.269999999997</v>
       </c>
       <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
+      <c r="U23" s="50" t="s">
+        <v>697</v>
+      </c>
+      <c r="V23" s="57" cm="1">
+        <f t="array" ref="V23">SUMIF(Region,"South",Sales)</f>
+        <v>303623.68999999994</v>
+      </c>
       <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
       <c r="AA23" s="1"/>
       <c r="AB23" s="1"/>
@@ -5126,11 +5250,14 @@
       <c r="R24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="1"/>
+      <c r="U24" s="50" t="s">
+        <v>698</v>
+      </c>
+      <c r="V24" s="57" cm="1">
+        <f t="array" ref="V24">SUMIF(Region,"East",Sales)</f>
+        <v>337881.26999999996</v>
+      </c>
       <c r="W24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
       <c r="AA24" s="1"/>
       <c r="AB24" s="1"/>
@@ -5191,11 +5318,14 @@
       <c r="R25" s="1"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
+      <c r="U25" s="50" t="s">
+        <v>699</v>
+      </c>
+      <c r="V25" s="57" cm="1">
+        <f t="array" ref="V25">SUMIF(Region,"West",Sales)</f>
+        <v>346200.06999999983</v>
+      </c>
       <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
       <c r="AA25" s="1"/>
       <c r="AB25" s="1"/>
@@ -5328,8 +5458,13 @@
         <v>498</v>
       </c>
       <c r="T27" s="1"/>
-      <c r="U27" s="1"/>
-      <c r="V27" s="1"/>
+      <c r="U27" s="50" t="s">
+        <v>700</v>
+      </c>
+      <c r="V27" s="57" cm="1">
+        <f t="array" ref="V27">COUNTIF(Region,"North")</f>
+        <v>124</v>
+      </c>
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
@@ -5390,7 +5525,7 @@
         <v>58</v>
       </c>
       <c r="Q28" s="1"/>
-      <c r="R28" s="60" t="s">
+      <c r="R28" s="50" t="s">
         <v>687</v>
       </c>
       <c r="S28" s="57">
@@ -5398,8 +5533,13 @@
         <v>149</v>
       </c>
       <c r="T28" s="1"/>
-      <c r="U28" s="1"/>
-      <c r="V28" s="1"/>
+      <c r="U28" s="50" t="s">
+        <v>701</v>
+      </c>
+      <c r="V28" s="57" cm="1">
+        <f t="array" ref="V28">COUNTIF(Region,"South")</f>
+        <v>124</v>
+      </c>
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
@@ -5460,7 +5600,7 @@
         <v>68</v>
       </c>
       <c r="Q29" s="1"/>
-      <c r="R29" s="60" t="s">
+      <c r="R29" s="50" t="s">
         <v>688</v>
       </c>
       <c r="S29" s="57">
@@ -5468,8 +5608,13 @@
         <v>164</v>
       </c>
       <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
-      <c r="V29" s="1"/>
+      <c r="U29" s="50" t="s">
+        <v>702</v>
+      </c>
+      <c r="V29" s="57" cm="1">
+        <f t="array" ref="V29">COUNTIF(Region,"East")</f>
+        <v>125</v>
+      </c>
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
@@ -5530,7 +5675,7 @@
         <v>41</v>
       </c>
       <c r="Q30" s="1"/>
-      <c r="R30" s="60" t="s">
+      <c r="R30" s="50" t="s">
         <v>689</v>
       </c>
       <c r="S30" s="57">
@@ -5538,8 +5683,13 @@
         <v>185</v>
       </c>
       <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="1"/>
+      <c r="U30" s="50" t="s">
+        <v>703</v>
+      </c>
+      <c r="V30" s="57" cm="1">
+        <f t="array" ref="V30">COUNTIF(Region,"West")</f>
+        <v>125</v>
+      </c>
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
@@ -5601,7 +5751,7 @@
       </c>
       <c r="Q31" s="1"/>
       <c r="R31" s="1"/>
-      <c r="S31" s="59"/>
+      <c r="S31" s="58"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
@@ -5665,7 +5815,7 @@
         <v>68</v>
       </c>
       <c r="Q32" s="1"/>
-      <c r="R32" s="60" t="s">
+      <c r="R32" s="50" t="s">
         <v>690</v>
       </c>
       <c r="S32" s="57" cm="1">
@@ -5735,7 +5885,7 @@
         <v>16</v>
       </c>
       <c r="Q33" s="1"/>
-      <c r="R33" s="60" t="s">
+      <c r="R33" s="50" t="s">
         <v>691</v>
       </c>
       <c r="S33" s="57" cm="1">
@@ -5805,7 +5955,7 @@
         <v>55</v>
       </c>
       <c r="Q34" s="1"/>
-      <c r="R34" s="60" t="s">
+      <c r="R34" s="50" t="s">
         <v>692</v>
       </c>
       <c r="S34" s="57" cm="1">
@@ -5875,7 +6025,7 @@
         <v>27</v>
       </c>
       <c r="Q35" s="1"/>
-      <c r="R35" s="60" t="s">
+      <c r="R35" s="50" t="s">
         <v>693</v>
       </c>
       <c r="S35" s="57" cm="1">
@@ -5945,7 +6095,7 @@
         <v>16</v>
       </c>
       <c r="Q36" s="1"/>
-      <c r="R36" s="60" t="s">
+      <c r="R36" s="50" t="s">
         <v>694</v>
       </c>
       <c r="S36" s="57" cm="1">
@@ -6080,10 +6230,10 @@
         <v>16</v>
       </c>
       <c r="Q38" s="1"/>
-      <c r="R38" s="58" t="s">
+      <c r="R38" s="50" t="s">
         <v>695</v>
       </c>
-      <c r="S38" s="1">
+      <c r="S38" s="57">
         <f>COUNTIFS(DMart_Sales_data[customer_type],"=Member",DMart_Sales_data[payment_mode],"=UPI")+COUNTIFS(DMart_Sales_data[customer_type],"=Member",DMart_Sales_data[payment_mode],"=Card")</f>
         <v>97</v>
       </c>
@@ -6151,10 +6301,7 @@
       </c>
       <c r="Q39" s="1"/>
       <c r="R39" s="1"/>
-      <c r="S39" s="1">
-        <f>COUNTIFS(DMart_Sales_data[customer_type],"Member",DMart_Sales_data[payment_mode],OR(UPI,Card))</f>
-        <v>0</v>
-      </c>
+      <c r="S39" s="1"/>
       <c r="T39" s="1"/>
       <c r="U39" s="1"/>
       <c r="V39" s="1"/>
@@ -50095,7 +50242,7 @@
       <c r="Z1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="F1:F1048576">
     <cfRule type="top10" dxfId="8" priority="3" bottom="1" rank="10"/>
     <cfRule type="top10" dxfId="7" priority="4" bottom="1" rank="10"/>
@@ -50269,7 +50416,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD2C2FD5-8379-4925-B2E3-1BBDDF1E9A2D}">
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:W45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -50281,9 +50428,12 @@
     <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.109375" customWidth="1"/>
     <col min="14" max="14" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.33203125" customWidth="1"/>
+    <col min="22" max="22" width="27" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" s="33" t="s">
         <v>576</v>
       </c>
@@ -50318,7 +50468,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="34" t="s">
         <v>577</v>
       </c>
@@ -50355,8 +50505,25 @@
         <f>IF(OR(K2&gt;=75,M2&gt;=75),"A+", "A")</f>
         <v>A+</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R2" s="33" t="s">
+        <v>576</v>
+      </c>
+      <c r="S2" s="33" t="s">
+        <v>584</v>
+      </c>
+      <c r="T2" s="35" t="s">
+        <v>707</v>
+      </c>
+      <c r="U2" s="35"/>
+      <c r="V2" s="33" t="s">
+        <v>708</v>
+      </c>
+      <c r="W2" s="60">
+        <f>COUNTIF(T3:T7,T4)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="34" t="s">
         <v>578</v>
       </c>
@@ -50390,11 +50557,20 @@
         <v>A</v>
       </c>
       <c r="O3" s="35" t="str">
-        <f>IF(OR(K3&gt;=75,M3&gt;=75),"A+DMartDataSet!S38", "A")</f>
-        <v>A+DMartDataSet!S38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+        <f>IF(OR(K3&gt;=75,M3&gt;=75),"A+", "A")</f>
+        <v>A+</v>
+      </c>
+      <c r="R3" s="34" t="s">
+        <v>577</v>
+      </c>
+      <c r="S3" s="34" t="s">
+        <v>585</v>
+      </c>
+      <c r="T3" s="35">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="34" t="s">
         <v>579</v>
       </c>
@@ -50431,8 +50607,17 @@
         <f>IF(OR(K4&gt;=75,M4&gt;=75),"A+", "A")</f>
         <v>A</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R4" s="34" t="s">
+        <v>578</v>
+      </c>
+      <c r="S4" s="34" t="s">
+        <v>586</v>
+      </c>
+      <c r="T4" s="35">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
         <v>580</v>
       </c>
@@ -50469,8 +50654,17 @@
         <f>IF(OR(K5&gt;=75,M5&gt;=75),"A+", "A")</f>
         <v>A+</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R5" s="34" t="s">
+        <v>579</v>
+      </c>
+      <c r="S5" s="34" t="s">
+        <v>587</v>
+      </c>
+      <c r="T5" s="35">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
         <v>2</v>
       </c>
@@ -50487,8 +50681,17 @@
         <f t="shared" si="0"/>
         <v>Not Achieved</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R6" s="34" t="s">
+        <v>580</v>
+      </c>
+      <c r="S6" s="34" t="s">
+        <v>588</v>
+      </c>
+      <c r="T6" s="35">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="34" t="s">
         <v>581</v>
       </c>
@@ -50505,20 +50708,31 @@
         <f t="shared" si="0"/>
         <v>Achieved</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R7" s="34"/>
+      <c r="S7" s="34"/>
+      <c r="T7" s="35">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
         <v>582</v>
       </c>
       <c r="B8" s="35"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R8" s="30"/>
+      <c r="S8" s="30"/>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
         <v>583</v>
       </c>
       <c r="B9" s="35"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="R9" s="30"/>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="R10" s="30"/>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D12" s="33" t="s">
         <v>584</v>
       </c>
@@ -50550,7 +50764,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D13" s="34" t="s">
         <v>585</v>
       </c>
@@ -50582,7 +50796,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D14" s="34" t="s">
         <v>586</v>
       </c>
@@ -50614,7 +50828,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D15" s="34" t="s">
         <v>587</v>
       </c>
@@ -50646,7 +50860,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="D16" s="34" t="s">
         <v>588</v>
       </c>
@@ -51127,7 +51341,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F2:G7">
     <sortCondition ref="F2:F7" customList="January,February,March,April,May,June,July,August,September,October,November,December"/>
   </sortState>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <conditionalFormatting sqref="G2:G7">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
       <formula>50000</formula>
@@ -51147,6 +51361,246 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{389844F2-09F9-438D-B186-7B9745B74C8A}">
+  <dimension ref="A2:J17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="31" t="s">
+        <v>711</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>606</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>577</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>637</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="35">
+        <v>1001</v>
+      </c>
+      <c r="B3" s="35" t="s">
+        <v>610</v>
+      </c>
+      <c r="C3" s="35">
+        <v>70000</v>
+      </c>
+      <c r="D3" s="35" t="str">
+        <f>IF(C3&gt;=$H$21,"10%",IF(C3&gt;=$H$22,"10%",IF(C3&gt;=$H$23,"5%","0%")))</f>
+        <v>10%</v>
+      </c>
+      <c r="E3" s="35">
+        <f>C3*D3</f>
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="35">
+        <v>1002</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>611</v>
+      </c>
+      <c r="C4" s="35">
+        <v>50000</v>
+      </c>
+      <c r="D4" s="35" t="str">
+        <f>IF(C4&gt;=$H$21,"5%",IF(C4&gt;=$H$22,"10%",IF(C4&gt;=$H$23,"5%","0%")))</f>
+        <v>5%</v>
+      </c>
+      <c r="E4" s="35">
+        <f>C4*D4</f>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="35">
+        <v>1003</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>612</v>
+      </c>
+      <c r="C5" s="35">
+        <v>45000</v>
+      </c>
+      <c r="D5" s="35" t="str">
+        <f>IF(C5&gt;=$H$21,"0%",IF(C5&gt;=$H$22,"10%",IF(C5&gt;=$H$23,"5%","0%")))</f>
+        <v>0%</v>
+      </c>
+      <c r="E5" s="35">
+        <f>C5*D5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="35">
+        <v>1004</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>613</v>
+      </c>
+      <c r="C6" s="35">
+        <v>75000</v>
+      </c>
+      <c r="D6" s="35" t="str">
+        <f>IF(C6&gt;=$H$21,"15%",IF(C6&gt;=$H$22,"10%",IF(C6&gt;=$H$23,"5%","0%")))</f>
+        <v>15%</v>
+      </c>
+      <c r="E6" s="35">
+        <f>C6*D6</f>
+        <v>11250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="35">
+        <v>1005</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>632</v>
+      </c>
+      <c r="C7" s="35">
+        <v>55000</v>
+      </c>
+      <c r="D7" s="35" t="str">
+        <f>IF(C7&gt;=$H$21,"5%",IF(C7&gt;=$H$22,"10%",IF(C7&gt;=$H$23,"5%","0%")))</f>
+        <v>5%</v>
+      </c>
+      <c r="E7" s="35">
+        <f>C7*D7</f>
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B10" s="64" t="s">
+        <v>712</v>
+      </c>
+      <c r="C10" s="64" t="s">
+        <v>577</v>
+      </c>
+      <c r="D10" s="64" t="s">
+        <v>638</v>
+      </c>
+      <c r="F10" s="63" t="s">
+        <v>713</v>
+      </c>
+      <c r="I10" t="s">
+        <v>577</v>
+      </c>
+      <c r="J10">
+        <f>VLOOKUP(B11,A3:E7,MATCH("Sales",A2:E2,0),FALSE)</f>
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B11" s="35">
+        <v>1004</v>
+      </c>
+      <c r="C11" s="35">
+        <f>VLOOKUP(B11,A3:C7,3,FALSE)</f>
+        <v>75000</v>
+      </c>
+      <c r="D11" s="35">
+        <f>VLOOKUP(B12,A4:E8,MATCH("Bonus Amount",A2:E2,0),FALSE)</f>
+        <v>2750</v>
+      </c>
+      <c r="F11">
+        <f>MATCH("Mangesh",B3:B7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="I11" t="s">
+        <v>638</v>
+      </c>
+      <c r="J11">
+        <f>VLOOKUP(B12,A4:E8,MATCH("Bonus Amount",A2:E2,0),FALSE)</f>
+        <v>2750</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B12" s="35">
+        <v>1005</v>
+      </c>
+      <c r="C12" s="35">
+        <f>VLOOKUP(B12,A4:C8,3,FALSE)</f>
+        <v>55000</v>
+      </c>
+      <c r="D12" s="35"/>
+      <c r="F12">
+        <f>MATCH("Mangesh",B4:B7,0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="65" t="s">
+        <v>716</v>
+      </c>
+      <c r="B14" s="66" t="s">
+        <v>715</v>
+      </c>
+      <c r="C14" s="66" t="s">
+        <v>714</v>
+      </c>
+      <c r="D14" s="66" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B15" s="35">
+        <v>1003</v>
+      </c>
+      <c r="C15" s="35">
+        <f>INDEX(A3:E7,3,3)</f>
+        <v>45000</v>
+      </c>
+      <c r="D15" s="35">
+        <f>INDEX(A3:E7,3,5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B16" s="35">
+        <v>1001</v>
+      </c>
+      <c r="C16" s="35">
+        <f>INDEX($A$3:$E$7,MATCH(B16,A3:A7,0),3)</f>
+        <v>70000</v>
+      </c>
+      <c r="D16" s="35" t="e" cm="1">
+        <f t="array" ref="D16">INDEX(A3:E7,MATCH(B16,A2:E2,0),FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B17" s="67">
+        <v>1003</v>
+      </c>
+      <c r="C17" s="35">
+        <f>INDEX(A4:E8,MATCH(B17,A4:A8,0),MATCH(C2,A2:E2,0))</f>
+        <v>45000</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11 B15:B16" xr:uid="{5DD0D1EB-1A92-41BA-A6DD-D0BAF7916F53}">
+      <formula1>$A$3:$A$7</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D630A1D-FB86-497E-A396-012A487AFACF}">
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -51244,83 +51698,124 @@
       <c r="F22" s="30"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A234BB-BD17-4FE0-89DF-BA7C71B4B0C1}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>596</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>604</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90A234BB-BD17-4FE0-89DF-BA7C71B4B0C1}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>593</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>595</v>
+      </c>
+      <c r="D4">
+        <v>120</v>
+      </c>
+      <c r="F4">
+        <f>SUBTOTAL(1,D4:D9)</f>
+        <v>96.333333333333329</v>
+      </c>
+      <c r="H4">
+        <f>SUBTOTAL(101,D4:D9)</f>
+        <v>96.333333333333329</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>598</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <f>SUBTOTAL(9,D4:D9)</f>
+        <v>578</v>
+      </c>
+      <c r="H5">
+        <f>SUBTOTAL(109,D4:D9)</f>
+        <v>578</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>596</v>
+      </c>
+      <c r="D6">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>600</v>
+      </c>
+      <c r="D7">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>601</v>
+      </c>
+      <c r="D8">
+        <v>45</v>
+      </c>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="61"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>602</v>
+      </c>
+      <c r="D9">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>604</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="D3:D9" xr:uid="{90A234BB-BD17-4FE0-89DF-BA7C71B4B0C1}"/>
+  <phoneticPr fontId="13" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9ADD8E7-B498-4D82-A60B-0B043A12DAA9}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -51418,7 +51913,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>